<commit_message>
Fuat Baslar Exercise 3A PART II
</commit_message>
<xml_diff>
--- a/Baslar_Ex3A_tables.xlsx
+++ b/Baslar_Ex3A_tables.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fb.baslar/Desktop/everything_about_python/Year-Up_DataAnalytics/week-02/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C17B908C-3847-F64D-B558-87F178EDFC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC42A1C8-5401-C745-9FE9-E3A3B8EB40D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12380" yWindow="6480" windowWidth="27240" windowHeight="16180" xr2:uid="{DB552174-F489-574B-AFB4-847CEC456262}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="4" xr2:uid="{DB552174-F489-574B-AFB4-847CEC456262}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Customers" sheetId="1" r:id="rId1"/>
+    <sheet name="Walkers" sheetId="2" r:id="rId2"/>
+    <sheet name="Dogs" sheetId="3" r:id="rId3"/>
+    <sheet name="Payments" sheetId="4" r:id="rId4"/>
+    <sheet name="Walks" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
   <si>
     <t>payment_id</t>
   </si>
@@ -51,13 +55,199 @@
   </si>
   <si>
     <t>payment_method</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>next_walk</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>adress</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>emergency_contact</t>
+  </si>
+  <si>
+    <t>walker_id</t>
+  </si>
+  <si>
+    <t>is_active</t>
+  </si>
+  <si>
+    <t>dog_id</t>
+  </si>
+  <si>
+    <t>dog_name</t>
+  </si>
+  <si>
+    <t>breed</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>walk_id</t>
+  </si>
+  <si>
+    <t>walk_date</t>
+  </si>
+  <si>
+    <t>walk_time</t>
+  </si>
+  <si>
+    <t>duration_minutes</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>555-1111</t>
+  </si>
+  <si>
+    <t>alice@walk.com</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>Jones</t>
+  </si>
+  <si>
+    <t>555-2222</t>
+  </si>
+  <si>
+    <t>bob@walk.com</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Johnson</t>
+  </si>
+  <si>
+    <t>555-0101</t>
+  </si>
+  <si>
+    <t>sarah.j@email.com</t>
+  </si>
+  <si>
+    <t>123 Maple St</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>Mike J. - 555-0102</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Park</t>
+  </si>
+  <si>
+    <t>555-0202</t>
+  </si>
+  <si>
+    <t>dpark@email.com</t>
+  </si>
+  <si>
+    <t>456 Oak Ave</t>
+  </si>
+  <si>
+    <t>Lisa Park - 555-0203</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>Gonzalez</t>
+  </si>
+  <si>
+    <t>555-0303</t>
+  </si>
+  <si>
+    <t>mgonzalez@email.com</t>
+  </si>
+  <si>
+    <t>789 Pine Rd</t>
+  </si>
+  <si>
+    <t>Evanston</t>
+  </si>
+  <si>
+    <t>Carlos G. - 555-0304</t>
+  </si>
+  <si>
+    <t>Buddy</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>German Shepherd</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>Poodle</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Venmo</t>
+  </si>
+  <si>
+    <t>Buddy was very energetic today.</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Walked in the big park.</t>
+  </si>
+  <si>
+    <t>Upcoming scheduled walk.</t>
+  </si>
+  <si>
+    <t>Pending</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -66,14 +256,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -82,20 +279,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,36 +311,43 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="5">
+    <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
+    <cellStyle name="40% - Accent6" xfId="4" builtinId="51"/>
+    <cellStyle name="60% - Accent1" xfId="2" builtinId="32"/>
+    <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -471,20 +680,319 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B320B9E8-5F8C-0742-BF19-4A371D4E8FB6}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
     <col min="2" max="2" width="15.5" customWidth="1"/>
-    <col min="4" max="4" width="15.5" customWidth="1"/>
-    <col min="5" max="5" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="11.5" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.5" customWidth="1"/>
+    <col min="11" max="11" width="19.5" customWidth="1"/>
+    <col min="12" max="12" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9286BC74-4D24-1747-BEFC-F5EBE1D25ECB}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84CDD59D-D629-F742-A94C-59D55EEC17FD}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>30.5</v>
+      </c>
+      <c r="F2" s="6">
+        <v>46132.375</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>35</v>
+      </c>
+      <c r="F3" s="6">
+        <v>46133.604166666664</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>12.5</v>
+      </c>
+      <c r="F4" s="6">
+        <v>46132.416666666664</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79841E6B-7D26-3B43-90AF-605F02000018}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -495,6 +1003,157 @@
       </c>
       <c r="E1" s="3" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>50</v>
+      </c>
+      <c r="D2" s="7">
+        <v>46127</v>
+      </c>
+      <c r="E2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1002</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>35</v>
+      </c>
+      <c r="D3" s="7">
+        <v>46128</v>
+      </c>
+      <c r="E3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF16BB08-23A5-FD4E-A5A6-30B040E83B36}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>5001</v>
+      </c>
+      <c r="B2">
+        <v>101</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7">
+        <v>46127</v>
+      </c>
+      <c r="E2" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="F2">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>5002</v>
+      </c>
+      <c r="B3">
+        <v>102</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7">
+        <v>46128</v>
+      </c>
+      <c r="E3" s="8">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F3">
+        <v>60</v>
+      </c>
+      <c r="G3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>5003</v>
+      </c>
+      <c r="B4">
+        <v>103</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7">
+        <v>46132</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F4">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>